<commit_message>
Fix Managed checkout form and record completed quality collection
</commit_message>
<xml_diff>
--- a/finance/VibeScroller-unit-economics.xlsx
+++ b/finance/VibeScroller-unit-economics.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R1bce08049cc94617"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="Re6d83dd854704778"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalogue" sheetId="3" r:id="Reb4ca799e0294c7a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario inputs" sheetId="4" r:id="Rf059950f0cd44b24"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="5" r:id="R657440d027494a6c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Volume" sheetId="6" r:id="Red9ba09d0dc74461"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Job estimate" sheetId="7" r:id="R6697db6bb61e458a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R0eac3e6a36ab41a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="R712d9f4865914d39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalogue" sheetId="3" r:id="Rd20d2df3cac743bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario inputs" sheetId="4" r:id="Rba27c16d877241fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="5" r:id="R8007def7266f4c61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Volume" sheetId="6" r:id="Rbdf4bbc486b2487f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Job estimate" sheetId="7" r:id="Rf69b54ff195e4c19"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -897,13 +897,18 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="6">
+  <x:numFmts count="11">
     <x:numFmt numFmtId="200" formatCode="0.000000;[Red](0.000000);&quot;-&quot;"/>
     <x:numFmt numFmtId="201" formatCode="0.0%;[Red](0.0%);&quot;-&quot;"/>
     <x:numFmt numFmtId="202" formatCode="€#,##0.00;[Red](€#,##0.00);&quot;-&quot;"/>
     <x:numFmt numFmtId="203" formatCode="#,##0;[Red](#,##0);&quot;-&quot;"/>
     <x:numFmt numFmtId="204" formatCode="#,##0.00;[Red](#,##0.00);&quot;-&quot;"/>
     <x:numFmt numFmtId="205" formatCode="0.0000;[Red](0.0000);&quot;-&quot;"/>
+    <x:numFmt numFmtId="206" formatCode="0.0%"/>
+    <x:numFmt numFmtId="207" formatCode="0.00"/>
+    <x:numFmt numFmtId="208" formatCode="�0.00"/>
+    <x:numFmt numFmtId="209" formatCode="0"/>
+    <x:numFmt numFmtId="210" formatCode="&quot;EUR &quot;#,##0.00"/>
   </x:numFmts>
   <x:fonts count="9">
     <x:font>
@@ -955,7 +960,7 @@
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="12">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -992,6 +997,26 @@
         <x:fgColor rgb="FFFFF8E7"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0E7490"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0E7490"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -1000,7 +1025,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="112">
+  <x:cellXfs count="132">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1177,6 +1202,48 @@
     <x:xf numFmtId="203" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="5" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="5" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="207" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="208" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="209" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="208" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="207" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="209" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="5" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="5" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="210" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="210" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -4640,7 +4707,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc504345a0555427c"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff5646ecc51d4f34"/>
 </x:worksheet>
 </file>
 
@@ -6746,13 +6813,25 @@
       <x:c r="AJ41" s="2"/>
       <x:c r="AK41" s="2"/>
     </x:row>
-    <x:row r="42" ht="20" customHeight="1">
-      <x:c r="A42" s="2"/>
-      <x:c r="B42" s="2"/>
-      <x:c r="C42" s="2"/>
-      <x:c r="D42" s="2"/>
-      <x:c r="E42" s="2"/>
-      <x:c r="F42" s="2"/>
+    <x:row r="42" ht="70" customHeight="1">
+      <x:c r="A42" s="30" t="str">
+        <x:v>managed payments rate</x:v>
+      </x:c>
+      <x:c r="B42" s="127" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C42" s="30" t="str">
+        <x:v>fraction of gross transaction amount including indirect tax</x:v>
+      </x:c>
+      <x:c r="D42" s="30" t="str">
+        <x:v>scenario</x:v>
+      </x:c>
+      <x:c r="E42" s="30" t="str">
+        <x:v>https://support.stripe.com/questions/managed-payments-pricing?locale=en-GB</x:v>
+      </x:c>
+      <x:c r="F42" s="30" t="str">
+        <x:v>Legacy direct-payment cases remain unchanged; selected Managed Payments cases use 3.5 percent in addition to payment and subscription Billing fees. Its indirect-tax handling is not added again as a separate Tax fee.</x:v>
+      </x:c>
       <x:c r="G42" s="2"/>
       <x:c r="H42" s="2"/>
       <x:c r="I42" s="2"/>
@@ -6785,13 +6864,25 @@
       <x:c r="AJ42" s="2"/>
       <x:c r="AK42" s="2"/>
     </x:row>
-    <x:row r="43" ht="20" customHeight="1">
-      <x:c r="A43" s="2"/>
-      <x:c r="B43" s="2"/>
-      <x:c r="C43" s="2"/>
-      <x:c r="D43" s="2"/>
-      <x:c r="E43" s="2"/>
-      <x:c r="F43" s="2"/>
+    <x:row r="43" ht="70" customHeight="1">
+      <x:c r="A43" s="30" t="str">
+        <x:v>radar screen ron</x:v>
+      </x:c>
+      <x:c r="B43" s="128" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C43" s="30" t="str">
+        <x:v>RON per screened transaction</x:v>
+      </x:c>
+      <x:c r="D43" s="30" t="str">
+        <x:v>scenario</x:v>
+      </x:c>
+      <x:c r="E43" s="30" t="str">
+        <x:v>Owner-authorized VibeScroller Radar Plus dashboard quote, October 3 2026</x:v>
+      </x:c>
+      <x:c r="F43" s="30" t="str">
+        <x:v>Managed Payments includes ordinary fraud handling; selected advanced country-rule configuration has a separately approved RON 0.31 screening quote.</x:v>
+      </x:c>
       <x:c r="G43" s="2"/>
       <x:c r="H43" s="2"/>
       <x:c r="I43" s="2"/>
@@ -6824,13 +6915,25 @@
       <x:c r="AJ43" s="2"/>
       <x:c r="AK43" s="2"/>
     </x:row>
-    <x:row r="44" ht="20" customHeight="1">
-      <x:c r="A44" s="2"/>
-      <x:c r="B44" s="2"/>
-      <x:c r="C44" s="2"/>
-      <x:c r="D44" s="2"/>
-      <x:c r="E44" s="2"/>
-      <x:c r="F44" s="2"/>
+    <x:row r="44" ht="70" customHeight="1">
+      <x:c r="A44" s="30" t="str">
+        <x:v>screened per payment</x:v>
+      </x:c>
+      <x:c r="B44" s="128" t="n">
+        <x:v>1.1</x:v>
+      </x:c>
+      <x:c r="C44" s="30" t="str">
+        <x:v>screened attempts per successful payment</x:v>
+      </x:c>
+      <x:c r="D44" s="30" t="str">
+        <x:v>assumption</x:v>
+      </x:c>
+      <x:c r="E44" s="30" t="str">
+        <x:v>Conservative planning assumption; not a provider observation</x:v>
+      </x:c>
+      <x:c r="F44" s="30" t="str">
+        <x:v>Include declined/uncompleted screening exposure. Replace using actual fee records.</x:v>
+      </x:c>
       <x:c r="G44" s="2"/>
       <x:c r="H44" s="2"/>
       <x:c r="I44" s="2"/>
@@ -7883,7 +7986,7 @@
     <x:mergeCell ref="A2:F2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4861383deab94f99"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6082b63c9df4e26"/>
 </x:worksheet>
 </file>
 
@@ -10717,7 +10820,7 @@
     <x:mergeCell ref="A9:G12"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R00e981e177be440d"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R00b2853a70ab47dc"/>
 </x:worksheet>
 </file>
 
@@ -10748,9 +10851,9 @@
     <x:col min="21" max="21" width="16" hidden="0" customWidth="1"/>
     <x:col min="22" max="22" width="16" hidden="0" customWidth="1"/>
     <x:col min="23" max="23" width="16" hidden="0" customWidth="1"/>
-    <x:col min="24" max="24" width="14" hidden="0" customWidth="1"/>
-    <x:col min="25" max="25" width="14" hidden="0" customWidth="1"/>
-    <x:col min="26" max="26" width="14" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="21" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="21" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="21" hidden="0" customWidth="1"/>
     <x:col min="27" max="27" width="14" hidden="0" customWidth="1"/>
     <x:col min="28" max="28" width="14" hidden="0" customWidth="1"/>
     <x:col min="29" max="29" width="14" hidden="0" customWidth="1"/>
@@ -10955,9 +11058,15 @@
       <x:c r="W4" s="16" t="str">
         <x:v>months year</x:v>
       </x:c>
-      <x:c r="X4" s="2"/>
-      <x:c r="Y4" s="2"/>
-      <x:c r="Z4" s="2"/>
+      <x:c r="X4" s="129" t="str">
+        <x:v>managed payments rate</x:v>
+      </x:c>
+      <x:c r="Y4" s="129" t="str">
+        <x:v>radar screen ron</x:v>
+      </x:c>
+      <x:c r="Z4" s="129" t="str">
+        <x:v>screened per payment</x:v>
+      </x:c>
       <x:c r="AA4" s="2"/>
       <x:c r="AB4" s="2"/>
       <x:c r="AC4" s="2"/>
@@ -11062,9 +11171,18 @@
         <x:f>'Assumptions'!$B$26</x:f>
         <x:v>12</x:v>
       </x:c>
-      <x:c r="X5" s="2"/>
-      <x:c r="Y5" s="2"/>
-      <x:c r="Z5" s="2"/>
+      <x:c r="X5" s="118" t="n">
+        <x:f>'Assumptions'!$B$42</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y5" s="119" t="n">
+        <x:f>'Assumptions'!$B$43</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Z5" s="119" t="n">
+        <x:f>'Assumptions'!$B$44</x:f>
+        <x:v>1.1</x:v>
+      </x:c>
       <x:c r="AA5" s="2"/>
       <x:c r="AB5" s="2"/>
       <x:c r="AC5" s="2"/>
@@ -11168,9 +11286,18 @@
         <x:f>'Assumptions'!$B$26</x:f>
         <x:v>12</x:v>
       </x:c>
-      <x:c r="X6" s="2"/>
-      <x:c r="Y6" s="2"/>
-      <x:c r="Z6" s="2"/>
+      <x:c r="X6" s="118" t="n">
+        <x:f>'Assumptions'!$B$42</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y6" s="119" t="n">
+        <x:f>'Assumptions'!$B$43</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Z6" s="119" t="n">
+        <x:f>'Assumptions'!$B$44</x:f>
+        <x:v>1.1</x:v>
+      </x:c>
       <x:c r="AA6" s="2"/>
       <x:c r="AB6" s="2"/>
       <x:c r="AC6" s="2"/>
@@ -11274,9 +11401,18 @@
         <x:f>'Assumptions'!$B$26</x:f>
         <x:v>12</x:v>
       </x:c>
-      <x:c r="X7" s="2"/>
-      <x:c r="Y7" s="2"/>
-      <x:c r="Z7" s="2"/>
+      <x:c r="X7" s="118" t="n">
+        <x:f>'Assumptions'!$B$42</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y7" s="119" t="n">
+        <x:f>'Assumptions'!$B$43</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Z7" s="119" t="n">
+        <x:f>'Assumptions'!$B$44</x:f>
+        <x:v>1.1</x:v>
+      </x:c>
       <x:c r="AA7" s="2"/>
       <x:c r="AB7" s="2"/>
       <x:c r="AC7" s="2"/>
@@ -11380,9 +11516,18 @@
         <x:f>'Assumptions'!$B$26</x:f>
         <x:v>12</x:v>
       </x:c>
-      <x:c r="X8" s="2"/>
-      <x:c r="Y8" s="2"/>
-      <x:c r="Z8" s="2"/>
+      <x:c r="X8" s="118" t="n">
+        <x:f>'Assumptions'!$B$42</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y8" s="119" t="n">
+        <x:f>'Assumptions'!$B$43</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Z8" s="119" t="n">
+        <x:f>'Assumptions'!$B$44</x:f>
+        <x:v>1.1</x:v>
+      </x:c>
       <x:c r="AA8" s="2"/>
       <x:c r="AB8" s="2"/>
       <x:c r="AC8" s="2"/>
@@ -11484,9 +11629,18 @@
         <x:f>'Assumptions'!$B$26</x:f>
         <x:v>12</x:v>
       </x:c>
-      <x:c r="X9" s="2"/>
-      <x:c r="Y9" s="2"/>
-      <x:c r="Z9" s="2"/>
+      <x:c r="X9" s="118" t="n">
+        <x:f>'Assumptions'!$B$42</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y9" s="119" t="n">
+        <x:f>'Assumptions'!$B$43</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Z9" s="119" t="n">
+        <x:f>'Assumptions'!$B$44</x:f>
+        <x:v>1.1</x:v>
+      </x:c>
       <x:c r="AA9" s="2"/>
       <x:c r="AB9" s="2"/>
       <x:c r="AC9" s="2"/>
@@ -11587,9 +11741,18 @@
         <x:f>'Assumptions'!$B$26</x:f>
         <x:v>12</x:v>
       </x:c>
-      <x:c r="X10" s="2"/>
-      <x:c r="Y10" s="2"/>
-      <x:c r="Z10" s="2"/>
+      <x:c r="X10" s="118" t="n">
+        <x:f>'Assumptions'!$B$42</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y10" s="119" t="n">
+        <x:f>'Assumptions'!$B$43</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Z10" s="119" t="n">
+        <x:f>'Assumptions'!$B$44</x:f>
+        <x:v>1.1</x:v>
+      </x:c>
       <x:c r="AA10" s="2"/>
       <x:c r="AB10" s="2"/>
       <x:c r="AC10" s="2"/>
@@ -11692,9 +11855,18 @@
         <x:f>'Assumptions'!$B$26</x:f>
         <x:v>12</x:v>
       </x:c>
-      <x:c r="X11" s="2"/>
-      <x:c r="Y11" s="2"/>
-      <x:c r="Z11" s="2"/>
+      <x:c r="X11" s="118" t="n">
+        <x:f>'Assumptions'!$B$42</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y11" s="119" t="n">
+        <x:f>'Assumptions'!$B$43</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Z11" s="119" t="n">
+        <x:f>'Assumptions'!$B$44</x:f>
+        <x:v>1.1</x:v>
+      </x:c>
       <x:c r="AA11" s="2"/>
       <x:c r="AB11" s="2"/>
       <x:c r="AC11" s="2"/>
@@ -11797,9 +11969,18 @@
         <x:f>'Assumptions'!$B$26</x:f>
         <x:v>12</x:v>
       </x:c>
-      <x:c r="X12" s="2"/>
-      <x:c r="Y12" s="2"/>
-      <x:c r="Z12" s="2"/>
+      <x:c r="X12" s="118" t="n">
+        <x:f>'Assumptions'!$B$42</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y12" s="119" t="n">
+        <x:f>'Assumptions'!$B$43</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Z12" s="119" t="n">
+        <x:f>'Assumptions'!$B$44</x:f>
+        <x:v>1.1</x:v>
+      </x:c>
       <x:c r="AA12" s="2"/>
       <x:c r="AB12" s="2"/>
       <x:c r="AC12" s="2"/>
@@ -11898,9 +12079,18 @@
         <x:f>'Assumptions'!$B$26</x:f>
         <x:v>12</x:v>
       </x:c>
-      <x:c r="X13" s="2"/>
-      <x:c r="Y13" s="2"/>
-      <x:c r="Z13" s="2"/>
+      <x:c r="X13" s="118" t="n">
+        <x:f>'Assumptions'!$B$42</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y13" s="119" t="n">
+        <x:f>'Assumptions'!$B$43</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Z13" s="119" t="n">
+        <x:f>'Assumptions'!$B$44</x:f>
+        <x:v>1.1</x:v>
+      </x:c>
       <x:c r="AA13" s="2"/>
       <x:c r="AB13" s="2"/>
       <x:c r="AC13" s="2"/>
@@ -12003,9 +12193,18 @@
         <x:f>'Assumptions'!$B$26</x:f>
         <x:v>12</x:v>
       </x:c>
-      <x:c r="X14" s="2"/>
-      <x:c r="Y14" s="2"/>
-      <x:c r="Z14" s="2"/>
+      <x:c r="X14" s="118" t="n">
+        <x:f>'Assumptions'!$B$42</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y14" s="119" t="n">
+        <x:f>'Assumptions'!$B$43</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Z14" s="119" t="n">
+        <x:f>'Assumptions'!$B$44</x:f>
+        <x:v>1.1</x:v>
+      </x:c>
       <x:c r="AA14" s="2"/>
       <x:c r="AB14" s="2"/>
       <x:c r="AC14" s="2"/>
@@ -12018,33 +12217,106 @@
       <x:c r="AJ14" s="2"/>
       <x:c r="AK14" s="2"/>
     </x:row>
-    <x:row r="15" ht="20" customHeight="1">
-      <x:c r="A15" s="2"/>
-      <x:c r="B15" s="2"/>
-      <x:c r="C15" s="2"/>
-      <x:c r="D15" s="2"/>
-      <x:c r="E15" s="2"/>
-      <x:c r="F15" s="2"/>
-      <x:c r="G15" s="2"/>
-      <x:c r="H15" s="2"/>
-      <x:c r="I15" s="2"/>
-      <x:c r="J15" s="2"/>
-      <x:c r="K15" s="2"/>
-      <x:c r="L15" s="2"/>
-      <x:c r="M15" s="2"/>
-      <x:c r="N15" s="2"/>
-      <x:c r="O15" s="2"/>
-      <x:c r="P15" s="2"/>
-      <x:c r="Q15" s="2"/>
-      <x:c r="R15" s="2"/>
-      <x:c r="S15" s="2"/>
-      <x:c r="T15" s="2"/>
-      <x:c r="U15" s="2"/>
-      <x:c r="V15" s="2"/>
-      <x:c r="W15" s="2"/>
-      <x:c r="X15" s="2"/>
-      <x:c r="Y15" s="2"/>
-      <x:c r="Z15" s="2"/>
+    <x:row r="15" ht="42" customHeight="1">
+      <x:c r="A15" s="30" t="str">
+        <x:v>Managed Payments launch, full allowance</x:v>
+      </x:c>
+      <x:c r="B15" s="2" t="n">
+        <x:f>'Assumptions'!$B$5</x:f>
+        <x:v>0.21</x:v>
+      </x:c>
+      <x:c r="C15" s="2" t="n">
+        <x:f>'Assumptions'!$B$6</x:f>
+        <x:v>0.02</x:v>
+      </x:c>
+      <x:c r="D15" s="2" t="n">
+        <x:f>'Assumptions'!$B$7</x:f>
+        <x:v>0.018</x:v>
+      </x:c>
+      <x:c r="E15" s="2" t="n">
+        <x:f>'Assumptions'!$B$8</x:f>
+        <x:v>0.007</x:v>
+      </x:c>
+      <x:c r="F15" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G15" s="2" t="n">
+        <x:f>'Assumptions'!$B$10</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H15" s="2" t="n">
+        <x:f>'Assumptions'!$B$11</x:f>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I15" s="2" t="n">
+        <x:f>'Assumptions'!$B$12</x:f>
+        <x:v>0.005</x:v>
+      </x:c>
+      <x:c r="J15" s="2" t="n">
+        <x:f>'Assumptions'!$B$13</x:f>
+        <x:v>0.001</x:v>
+      </x:c>
+      <x:c r="K15" s="2" t="n">
+        <x:f>'Assumptions'!$B$14</x:f>
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="L15" s="2" t="n">
+        <x:f>'Assumptions'!$B$15</x:f>
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="M15" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N15" s="2" t="n">
+        <x:f>'Assumptions'!$B$17</x:f>
+        <x:v>0.55</x:v>
+      </x:c>
+      <x:c r="O15" s="2" t="n">
+        <x:f>'Assumptions'!$B$18</x:f>
+        <x:v>0.95</x:v>
+      </x:c>
+      <x:c r="P15" s="2" t="n">
+        <x:f>'Assumptions'!$B$19</x:f>
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="Q15" s="2" t="n">
+        <x:f>'Assumptions'!$B$20</x:f>
+        <x:v>0.7</x:v>
+      </x:c>
+      <x:c r="R15" s="2" t="n">
+        <x:f>'Assumptions'!$B$21</x:f>
+        <x:v>0.15</x:v>
+      </x:c>
+      <x:c r="S15" s="2" t="n">
+        <x:f>'Assumptions'!$B$22</x:f>
+        <x:v>0.65</x:v>
+      </x:c>
+      <x:c r="T15" s="2" t="n">
+        <x:f>'Assumptions'!$B$23</x:f>
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="U15" s="2" t="n">
+        <x:f>'Assumptions'!$B$24</x:f>
+        <x:v>365.25</x:v>
+      </x:c>
+      <x:c r="V15" s="2" t="n">
+        <x:f>'Assumptions'!$B$25</x:f>
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="W15" s="2" t="n">
+        <x:f>'Assumptions'!$B$26</x:f>
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="X15" s="118" t="n">
+        <x:v>0.035</x:v>
+      </x:c>
+      <x:c r="Y15" s="119" t="n">
+        <x:v>0.31</x:v>
+      </x:c>
+      <x:c r="Z15" s="119" t="n">
+        <x:f>'Assumptions'!$B$44</x:f>
+        <x:v>1.1</x:v>
+      </x:c>
       <x:c r="AA15" s="2"/>
       <x:c r="AB15" s="2"/>
       <x:c r="AC15" s="2"/>
@@ -12057,33 +12329,104 @@
       <x:c r="AJ15" s="2"/>
       <x:c r="AK15" s="2"/>
     </x:row>
-    <x:row r="16" ht="20" customHeight="1">
-      <x:c r="A16" s="2"/>
-      <x:c r="B16" s="2"/>
-      <x:c r="C16" s="2"/>
-      <x:c r="D16" s="2"/>
-      <x:c r="E16" s="2"/>
-      <x:c r="F16" s="2"/>
-      <x:c r="G16" s="2"/>
-      <x:c r="H16" s="2"/>
-      <x:c r="I16" s="2"/>
-      <x:c r="J16" s="2"/>
-      <x:c r="K16" s="2"/>
-      <x:c r="L16" s="2"/>
-      <x:c r="M16" s="2"/>
-      <x:c r="N16" s="2"/>
-      <x:c r="O16" s="2"/>
-      <x:c r="P16" s="2"/>
-      <x:c r="Q16" s="2"/>
-      <x:c r="R16" s="2"/>
-      <x:c r="S16" s="2"/>
-      <x:c r="T16" s="2"/>
-      <x:c r="U16" s="2"/>
-      <x:c r="V16" s="2"/>
-      <x:c r="W16" s="2"/>
-      <x:c r="X16" s="2"/>
-      <x:c r="Y16" s="2"/>
-      <x:c r="Z16" s="2"/>
+    <x:row r="16" ht="42" customHeight="1">
+      <x:c r="A16" s="30" t="str">
+        <x:v>Managed Payments all annual, full allowance</x:v>
+      </x:c>
+      <x:c r="B16" s="2" t="n">
+        <x:f>'Assumptions'!$B$5</x:f>
+        <x:v>0.21</x:v>
+      </x:c>
+      <x:c r="C16" s="2" t="n">
+        <x:f>'Assumptions'!$B$6</x:f>
+        <x:v>0.02</x:v>
+      </x:c>
+      <x:c r="D16" s="2" t="n">
+        <x:f>'Assumptions'!$B$7</x:f>
+        <x:v>0.018</x:v>
+      </x:c>
+      <x:c r="E16" s="2" t="n">
+        <x:f>'Assumptions'!$B$8</x:f>
+        <x:v>0.007</x:v>
+      </x:c>
+      <x:c r="F16" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G16" s="2" t="n">
+        <x:f>'Assumptions'!$B$10</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H16" s="2" t="n">
+        <x:f>'Assumptions'!$B$11</x:f>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I16" s="2" t="n">
+        <x:f>'Assumptions'!$B$12</x:f>
+        <x:v>0.005</x:v>
+      </x:c>
+      <x:c r="J16" s="2" t="n">
+        <x:f>'Assumptions'!$B$13</x:f>
+        <x:v>0.001</x:v>
+      </x:c>
+      <x:c r="K16" s="2" t="n">
+        <x:f>'Assumptions'!$B$14</x:f>
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="L16" s="2" t="n">
+        <x:f>'Assumptions'!$B$15</x:f>
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="M16" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N16" s="2" t="n">
+        <x:f>'Assumptions'!$B$17</x:f>
+        <x:v>0.55</x:v>
+      </x:c>
+      <x:c r="O16" s="2" t="n">
+        <x:f>'Assumptions'!$B$18</x:f>
+        <x:v>0.95</x:v>
+      </x:c>
+      <x:c r="P16" s="2" t="n">
+        <x:f>'Assumptions'!$B$19</x:f>
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="Q16" s="2" t="n">
+        <x:f>'Assumptions'!$B$20</x:f>
+        <x:v>0.7</x:v>
+      </x:c>
+      <x:c r="R16" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S16" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T16" s="2" t="n">
+        <x:f>'Assumptions'!$B$23</x:f>
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="U16" s="2" t="n">
+        <x:f>'Assumptions'!$B$24</x:f>
+        <x:v>365.25</x:v>
+      </x:c>
+      <x:c r="V16" s="2" t="n">
+        <x:f>'Assumptions'!$B$25</x:f>
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="W16" s="2" t="n">
+        <x:f>'Assumptions'!$B$26</x:f>
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="X16" s="118" t="n">
+        <x:v>0.035</x:v>
+      </x:c>
+      <x:c r="Y16" s="119" t="n">
+        <x:v>0.31</x:v>
+      </x:c>
+      <x:c r="Z16" s="119" t="n">
+        <x:f>'Assumptions'!$B$44</x:f>
+        <x:v>1.1</x:v>
+      </x:c>
       <x:c r="AA16" s="2"/>
       <x:c r="AB16" s="2"/>
       <x:c r="AC16" s="2"/>
@@ -12096,33 +12439,103 @@
       <x:c r="AJ16" s="2"/>
       <x:c r="AK16" s="2"/>
     </x:row>
-    <x:row r="17" ht="20" customHeight="1">
-      <x:c r="A17" s="2"/>
-      <x:c r="B17" s="2"/>
-      <x:c r="C17" s="2"/>
-      <x:c r="D17" s="2"/>
-      <x:c r="E17" s="2"/>
-      <x:c r="F17" s="2"/>
-      <x:c r="G17" s="2"/>
-      <x:c r="H17" s="2"/>
-      <x:c r="I17" s="2"/>
-      <x:c r="J17" s="2"/>
-      <x:c r="K17" s="2"/>
-      <x:c r="L17" s="2"/>
-      <x:c r="M17" s="2"/>
-      <x:c r="N17" s="2"/>
-      <x:c r="O17" s="2"/>
-      <x:c r="P17" s="2"/>
-      <x:c r="Q17" s="2"/>
-      <x:c r="R17" s="2"/>
-      <x:c r="S17" s="2"/>
-      <x:c r="T17" s="2"/>
-      <x:c r="U17" s="2"/>
-      <x:c r="V17" s="2"/>
-      <x:c r="W17" s="2"/>
-      <x:c r="X17" s="2"/>
-      <x:c r="Y17" s="2"/>
-      <x:c r="Z17" s="2"/>
+    <x:row r="17" ht="42" customHeight="1">
+      <x:c r="A17" s="30" t="str">
+        <x:v>Managed Payments Starter annual, full allowance</x:v>
+      </x:c>
+      <x:c r="B17" s="2" t="n">
+        <x:f>'Assumptions'!$B$5</x:f>
+        <x:v>0.21</x:v>
+      </x:c>
+      <x:c r="C17" s="2" t="n">
+        <x:f>'Assumptions'!$B$6</x:f>
+        <x:v>0.02</x:v>
+      </x:c>
+      <x:c r="D17" s="2" t="n">
+        <x:f>'Assumptions'!$B$7</x:f>
+        <x:v>0.018</x:v>
+      </x:c>
+      <x:c r="E17" s="2" t="n">
+        <x:f>'Assumptions'!$B$8</x:f>
+        <x:v>0.007</x:v>
+      </x:c>
+      <x:c r="F17" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G17" s="2" t="n">
+        <x:f>'Assumptions'!$B$10</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H17" s="2" t="n">
+        <x:f>'Assumptions'!$B$11</x:f>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I17" s="2" t="n">
+        <x:f>'Assumptions'!$B$12</x:f>
+        <x:v>0.005</x:v>
+      </x:c>
+      <x:c r="J17" s="2" t="n">
+        <x:f>'Assumptions'!$B$13</x:f>
+        <x:v>0.001</x:v>
+      </x:c>
+      <x:c r="K17" s="2" t="n">
+        <x:f>'Assumptions'!$B$14</x:f>
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="L17" s="2" t="n">
+        <x:f>'Assumptions'!$B$15</x:f>
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="M17" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N17" s="2" t="n">
+        <x:f>'Assumptions'!$B$17</x:f>
+        <x:v>0.55</x:v>
+      </x:c>
+      <x:c r="O17" s="2" t="n">
+        <x:f>'Assumptions'!$B$18</x:f>
+        <x:v>0.95</x:v>
+      </x:c>
+      <x:c r="P17" s="2" t="n">
+        <x:f>'Assumptions'!$B$19</x:f>
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="Q17" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="R17" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S17" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T17" s="2" t="n">
+        <x:f>'Assumptions'!$B$23</x:f>
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="U17" s="2" t="n">
+        <x:f>'Assumptions'!$B$24</x:f>
+        <x:v>365.25</x:v>
+      </x:c>
+      <x:c r="V17" s="2" t="n">
+        <x:f>'Assumptions'!$B$25</x:f>
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="W17" s="2" t="n">
+        <x:f>'Assumptions'!$B$26</x:f>
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="X17" s="118" t="n">
+        <x:v>0.035</x:v>
+      </x:c>
+      <x:c r="Y17" s="119" t="n">
+        <x:v>0.31</x:v>
+      </x:c>
+      <x:c r="Z17" s="119" t="n">
+        <x:f>'Assumptions'!$B$44</x:f>
+        <x:v>1.1</x:v>
+      </x:c>
       <x:c r="AA17" s="2"/>
       <x:c r="AB17" s="2"/>
       <x:c r="AC17" s="2"/>
@@ -14208,7 +14621,7 @@
     <x:mergeCell ref="A2:W2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c7fa32ee9b1469d"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R069ed78bd7b44830"/>
 </x:worksheet>
 </file>
 
@@ -14478,11 +14891,11 @@
         <x:v>0.67</x:v>
       </x:c>
       <x:c r="H5" s="44" t="n">
-        <x:f>B5*('Scenario inputs'!$D$5+'Scenario inputs'!$E$5+'Scenario inputs'!$F$5)</x:f>
+        <x:f>B5*('Scenario inputs'!$D$5+'Scenario inputs'!$E$5+'Scenario inputs'!$F$5+'Scenario inputs'!$X$5)</x:f>
         <x:v>0.7649266517857142</x:v>
       </x:c>
       <x:c r="I5" s="44" t="n">
-        <x:f>D5*'Scenario inputs'!$G$5/'Scenario inputs'!$H$5</x:f>
+        <x:f>D5*('Scenario inputs'!$G$5+'Scenario inputs'!$Y$5*'Scenario inputs'!$Z$5)/'Scenario inputs'!$H$5</x:f>
         <x:v>0.2637797619047619</x:v>
       </x:c>
       <x:c r="J5" s="44" t="n">
@@ -14567,11 +14980,11 @@
         <x:v>0.67</x:v>
       </x:c>
       <x:c r="H6" s="44" t="n">
-        <x:f>B6*('Scenario inputs'!$D$6+'Scenario inputs'!$E$6+'Scenario inputs'!$F$6)</x:f>
+        <x:f>B6*('Scenario inputs'!$D$6+'Scenario inputs'!$E$6+'Scenario inputs'!$F$6+'Scenario inputs'!$X$6)</x:f>
         <x:v>0.7649266517857142</x:v>
       </x:c>
       <x:c r="I6" s="44" t="n">
-        <x:f>D6*'Scenario inputs'!$G$6/'Scenario inputs'!$H$6</x:f>
+        <x:f>D6*('Scenario inputs'!$G$6+'Scenario inputs'!$Y$6*'Scenario inputs'!$Z$6)/'Scenario inputs'!$H$6</x:f>
         <x:v>0.2637797619047619</x:v>
       </x:c>
       <x:c r="J6" s="44" t="n">
@@ -14656,11 +15069,11 @@
         <x:v>0.67</x:v>
       </x:c>
       <x:c r="H7" s="44" t="n">
-        <x:f>B7*('Scenario inputs'!$D$7+'Scenario inputs'!$E$7+'Scenario inputs'!$F$7)</x:f>
+        <x:f>B7*('Scenario inputs'!$D$7+'Scenario inputs'!$E$7+'Scenario inputs'!$F$7+'Scenario inputs'!$X$7)</x:f>
         <x:v>0.7649266517857142</x:v>
       </x:c>
       <x:c r="I7" s="44" t="n">
-        <x:f>D7*'Scenario inputs'!$G$7/'Scenario inputs'!$H$7</x:f>
+        <x:f>D7*('Scenario inputs'!$G$7+'Scenario inputs'!$Y$7*'Scenario inputs'!$Z$7)/'Scenario inputs'!$H$7</x:f>
         <x:v>0.2637797619047619</x:v>
       </x:c>
       <x:c r="J7" s="44" t="n">
@@ -14745,11 +15158,11 @@
         <x:v>0.67</x:v>
       </x:c>
       <x:c r="H8" s="44" t="n">
-        <x:f>B8*('Scenario inputs'!$D$8+'Scenario inputs'!$E$8+'Scenario inputs'!$F$8)</x:f>
+        <x:f>B8*('Scenario inputs'!$D$8+'Scenario inputs'!$E$8+'Scenario inputs'!$F$8+'Scenario inputs'!$X$8)</x:f>
         <x:v>0.7649266517857142</x:v>
       </x:c>
       <x:c r="I8" s="44" t="n">
-        <x:f>D8*'Scenario inputs'!$G$8/'Scenario inputs'!$H$8</x:f>
+        <x:f>D8*('Scenario inputs'!$G$8+'Scenario inputs'!$Y$8*'Scenario inputs'!$Z$8)/'Scenario inputs'!$H$8</x:f>
         <x:v>0.2637797619047619</x:v>
       </x:c>
       <x:c r="J8" s="44" t="n">
@@ -14834,11 +15247,11 @@
         <x:v>0.67</x:v>
       </x:c>
       <x:c r="H9" s="44" t="n">
-        <x:f>B9*('Scenario inputs'!$D$9+'Scenario inputs'!$E$9+'Scenario inputs'!$F$9)</x:f>
+        <x:f>B9*('Scenario inputs'!$D$9+'Scenario inputs'!$E$9+'Scenario inputs'!$F$9+'Scenario inputs'!$X$9)</x:f>
         <x:v>0.625</x:v>
       </x:c>
       <x:c r="I9" s="44" t="n">
-        <x:f>D9*'Scenario inputs'!$G$9/'Scenario inputs'!$H$9</x:f>
+        <x:f>D9*('Scenario inputs'!$G$9+'Scenario inputs'!$Y$9*'Scenario inputs'!$Z$9)/'Scenario inputs'!$H$9</x:f>
         <x:v>0.016666666666666666</x:v>
       </x:c>
       <x:c r="J9" s="44" t="n">
@@ -14923,11 +15336,11 @@
         <x:v>0.55</x:v>
       </x:c>
       <x:c r="H10" s="44" t="n">
-        <x:f>B10*('Scenario inputs'!$D$10+'Scenario inputs'!$E$10+'Scenario inputs'!$F$10)</x:f>
+        <x:f>B10*('Scenario inputs'!$D$10+'Scenario inputs'!$E$10+'Scenario inputs'!$F$10+'Scenario inputs'!$X$10)</x:f>
         <x:v>0.475</x:v>
       </x:c>
       <x:c r="I10" s="44" t="n">
-        <x:f>D10*'Scenario inputs'!$G$10/'Scenario inputs'!$H$10</x:f>
+        <x:f>D10*('Scenario inputs'!$G$10+'Scenario inputs'!$Y$10*'Scenario inputs'!$Z$10)/'Scenario inputs'!$H$10</x:f>
         <x:v>0.016666666666666666</x:v>
       </x:c>
       <x:c r="J10" s="44" t="n">
@@ -15012,11 +15425,11 @@
         <x:v>0.67</x:v>
       </x:c>
       <x:c r="H11" s="44" t="n">
-        <x:f>B11*('Scenario inputs'!$D$11+'Scenario inputs'!$E$11+'Scenario inputs'!$F$11)</x:f>
+        <x:f>B11*('Scenario inputs'!$D$11+'Scenario inputs'!$E$11+'Scenario inputs'!$F$11+'Scenario inputs'!$X$11)</x:f>
         <x:v>0.6374388764880952</x:v>
       </x:c>
       <x:c r="I11" s="44" t="n">
-        <x:f>D11*'Scenario inputs'!$G$11/'Scenario inputs'!$H$11</x:f>
+        <x:f>D11*('Scenario inputs'!$G$11+'Scenario inputs'!$Y$11*'Scenario inputs'!$Z$11)/'Scenario inputs'!$H$11</x:f>
         <x:v>0.2637797619047619</x:v>
       </x:c>
       <x:c r="J11" s="44" t="n">
@@ -15101,11 +15514,11 @@
         <x:v>0.67</x:v>
       </x:c>
       <x:c r="H12" s="44" t="n">
-        <x:f>B12*('Scenario inputs'!$D$12+'Scenario inputs'!$E$12+'Scenario inputs'!$F$12)</x:f>
+        <x:f>B12*('Scenario inputs'!$D$12+'Scenario inputs'!$E$12+'Scenario inputs'!$F$12+'Scenario inputs'!$X$12)</x:f>
         <x:v>0.7649266517857142</x:v>
       </x:c>
       <x:c r="I12" s="44" t="n">
-        <x:f>D12*'Scenario inputs'!$G$12/'Scenario inputs'!$H$12</x:f>
+        <x:f>D12*('Scenario inputs'!$G$12+'Scenario inputs'!$Y$12*'Scenario inputs'!$Z$12)/'Scenario inputs'!$H$12</x:f>
         <x:v>0.2637797619047619</x:v>
       </x:c>
       <x:c r="J12" s="44" t="n">
@@ -15190,11 +15603,11 @@
         <x:v>1.9700000000000002</x:v>
       </x:c>
       <x:c r="H13" s="44" t="n">
-        <x:f>B13*('Scenario inputs'!$D$13+'Scenario inputs'!$E$13+'Scenario inputs'!$F$13)</x:f>
+        <x:f>B13*('Scenario inputs'!$D$13+'Scenario inputs'!$E$13+'Scenario inputs'!$F$13+'Scenario inputs'!$X$13)</x:f>
         <x:v>1.1091436450892855</x:v>
       </x:c>
       <x:c r="I13" s="44" t="n">
-        <x:f>D13*'Scenario inputs'!$G$13/'Scenario inputs'!$H$13</x:f>
+        <x:f>D13*('Scenario inputs'!$G$13+'Scenario inputs'!$Y$13*'Scenario inputs'!$Z$13)/'Scenario inputs'!$H$13</x:f>
         <x:v>0.2637797619047619</x:v>
       </x:c>
       <x:c r="J13" s="44" t="n">
@@ -15279,11 +15692,11 @@
         <x:v>0.67</x:v>
       </x:c>
       <x:c r="H14" s="44" t="n">
-        <x:f>B14*('Scenario inputs'!$D$14+'Scenario inputs'!$E$14+'Scenario inputs'!$F$14)</x:f>
+        <x:f>B14*('Scenario inputs'!$D$14+'Scenario inputs'!$E$14+'Scenario inputs'!$F$14+'Scenario inputs'!$X$14)</x:f>
         <x:v>0.7649266517857142</x:v>
       </x:c>
       <x:c r="I14" s="44" t="n">
-        <x:f>D14*'Scenario inputs'!$G$14/'Scenario inputs'!$H$14</x:f>
+        <x:f>D14*('Scenario inputs'!$G$14+'Scenario inputs'!$Y$14*'Scenario inputs'!$Z$14)/'Scenario inputs'!$H$14</x:f>
         <x:v>0.2637797619047619</x:v>
       </x:c>
       <x:c r="J14" s="44" t="n">
@@ -15339,24 +15752,74 @@
       <x:c r="AJ14" s="2"/>
       <x:c r="AK14" s="2"/>
     </x:row>
-    <x:row r="15" ht="20" customHeight="1">
-      <x:c r="A15" s="2"/>
-      <x:c r="B15" s="2"/>
-      <x:c r="C15" s="2"/>
-      <x:c r="D15" s="2"/>
-      <x:c r="E15" s="2"/>
-      <x:c r="F15" s="2"/>
-      <x:c r="G15" s="2"/>
-      <x:c r="H15" s="2"/>
-      <x:c r="I15" s="2"/>
-      <x:c r="J15" s="2"/>
-      <x:c r="K15" s="2"/>
-      <x:c r="L15" s="2"/>
-      <x:c r="M15" s="2"/>
-      <x:c r="N15" s="2"/>
-      <x:c r="O15" s="2"/>
-      <x:c r="P15" s="2"/>
-      <x:c r="Q15" s="2"/>
+    <x:row r="15" ht="42" customHeight="1">
+      <x:c r="A15" s="30" t="str">
+        <x:v>Managed Payments launch, full allowance</x:v>
+      </x:c>
+      <x:c r="B15" s="130" t="n">
+        <x:f>'Scenario inputs'!$Q$15*('Scenario inputs'!$R$15*'Catalogue'!$B$5*('Scenario inputs'!$U$15/'Scenario inputs'!$V$15/'Scenario inputs'!$W$15)+'Scenario inputs'!$S$15*'Catalogue'!$C$5+(1-'Scenario inputs'!$R$15-'Scenario inputs'!$S$15)*'Catalogue'!$D$5/'Scenario inputs'!$W$15)+(1-'Scenario inputs'!$Q$15)*('Scenario inputs'!$R$15*'Catalogue'!$B$6*('Scenario inputs'!$U$15/'Scenario inputs'!$V$15/'Scenario inputs'!$W$15)+'Scenario inputs'!$S$15*'Catalogue'!$C$6+(1-'Scenario inputs'!$R$15-'Scenario inputs'!$S$15)*'Catalogue'!$D$6/'Scenario inputs'!$W$15)</x:f>
+        <x:v>25.49755505952381</x:v>
+      </x:c>
+      <x:c r="C15" s="130" t="n">
+        <x:f>B15*(1-'Scenario inputs'!$C$15)/(1+'Scenario inputs'!$B$15)</x:f>
+        <x:v>20.650912362258953</x:v>
+      </x:c>
+      <x:c r="D15" s="123" t="n">
+        <x:f>'Scenario inputs'!$R$15*('Scenario inputs'!$U$15/'Scenario inputs'!$V$15/'Scenario inputs'!$W$15)+'Scenario inputs'!$S$15+(1-'Scenario inputs'!$R$15-'Scenario inputs'!$S$15)/'Scenario inputs'!$W$15</x:f>
+        <x:v>1.3188988095238094</x:v>
+      </x:c>
+      <x:c r="E15" s="124" t="n">
+        <x:f>'Scenario inputs'!$Q$15*('Scenario inputs'!$R$15*'Catalogue'!$E$5*('Scenario inputs'!$U$15/'Scenario inputs'!$V$15/'Scenario inputs'!$W$15)+(1-'Scenario inputs'!$R$15)*'Catalogue'!$F$5)+(1-'Scenario inputs'!$Q$15)*('Scenario inputs'!$R$15*'Catalogue'!$E$6*('Scenario inputs'!$U$15/'Scenario inputs'!$V$15/'Scenario inputs'!$W$15)+(1-'Scenario inputs'!$R$15)*'Catalogue'!$F$6)</x:f>
+        <x:v>360.7770089285715</x:v>
+      </x:c>
+      <x:c r="F15" s="130" t="n">
+        <x:f>E15*'Scenario inputs'!$L$15*'Scenario inputs'!$M$15</x:f>
+        <x:v>3.607770089285715</x:v>
+      </x:c>
+      <x:c r="G15" s="130" t="n">
+        <x:f>'Scenario inputs'!$Q$15*'Scenario inputs'!$N$15+(1-'Scenario inputs'!$Q$15)*'Scenario inputs'!$O$15</x:f>
+        <x:v>0.67</x:v>
+      </x:c>
+      <x:c r="H15" s="130" t="n">
+        <x:f>B15*('Scenario inputs'!$D$15+'Scenario inputs'!$E$15+'Scenario inputs'!$F$15+'Scenario inputs'!$X$15)</x:f>
+        <x:v>1.5298533035714283</x:v>
+      </x:c>
+      <x:c r="I15" s="130" t="n">
+        <x:f>D15*('Scenario inputs'!$G$15+'Scenario inputs'!$Y$15*'Scenario inputs'!$Z$15)/'Scenario inputs'!$H$15</x:f>
+        <x:v>0.35372866071428566</x:v>
+      </x:c>
+      <x:c r="J15" s="130" t="n">
+        <x:f>B15*'Scenario inputs'!$I$15</x:f>
+        <x:v>0.12748777529761904</x:v>
+      </x:c>
+      <x:c r="K15" s="130" t="n">
+        <x:f>D15*'Scenario inputs'!$J$15*'Scenario inputs'!$K$15</x:f>
+        <x:v>0.02637797619047619</x:v>
+      </x:c>
+      <x:c r="L15" s="131" t="n">
+        <x:f>SUM(F15:K15)</x:f>
+        <x:v>6.3152178050595245</x:v>
+      </x:c>
+      <x:c r="M15" s="131" t="n">
+        <x:f>C15-L15</x:f>
+        <x:v>14.335694557199428</x:v>
+      </x:c>
+      <x:c r="N15" s="130" t="n">
+        <x:f>'Scenario inputs'!$P$15</x:f>
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="O15" s="124" t="n">
+        <x:f>IF(M15&lt;=0,"Not attainable",MAX(1,ROUNDUP(N15/M15,0)))</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="P15" s="124" t="n">
+        <x:f>IF(C15*(1-'Scenario inputs'!$T$15)-L15&lt;=0,"Not attainable",MAX(1,ROUNDUP(N15/(C15*(1-'Scenario inputs'!$T$15)-L15),0)))</x:f>
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="Q15" s="118" t="n">
+        <x:f>IF(C15=0,"Not defined",M15/C15)</x:f>
+        <x:v>0.6941918258003436</x:v>
+      </x:c>
       <x:c r="R15" s="2"/>
       <x:c r="S15" s="2"/>
       <x:c r="T15" s="2"/>
@@ -15378,24 +15841,74 @@
       <x:c r="AJ15" s="2"/>
       <x:c r="AK15" s="2"/>
     </x:row>
-    <x:row r="16" ht="20" customHeight="1">
-      <x:c r="A16" s="2"/>
-      <x:c r="B16" s="2"/>
-      <x:c r="C16" s="2"/>
-      <x:c r="D16" s="2"/>
-      <x:c r="E16" s="2"/>
-      <x:c r="F16" s="2"/>
-      <x:c r="G16" s="2"/>
-      <x:c r="H16" s="2"/>
-      <x:c r="I16" s="2"/>
-      <x:c r="J16" s="2"/>
-      <x:c r="K16" s="2"/>
-      <x:c r="L16" s="2"/>
-      <x:c r="M16" s="2"/>
-      <x:c r="N16" s="2"/>
-      <x:c r="O16" s="2"/>
-      <x:c r="P16" s="2"/>
-      <x:c r="Q16" s="2"/>
+    <x:row r="16" ht="42" customHeight="1">
+      <x:c r="A16" s="30" t="str">
+        <x:v>Managed Payments all annual, full allowance</x:v>
+      </x:c>
+      <x:c r="B16" s="130" t="n">
+        <x:f>'Scenario inputs'!$Q$16*('Scenario inputs'!$R$16*'Catalogue'!$B$5*('Scenario inputs'!$U$16/'Scenario inputs'!$V$16/'Scenario inputs'!$W$16)+'Scenario inputs'!$S$16*'Catalogue'!$C$5+(1-'Scenario inputs'!$R$16-'Scenario inputs'!$S$16)*'Catalogue'!$D$5/'Scenario inputs'!$W$16)+(1-'Scenario inputs'!$Q$16)*('Scenario inputs'!$R$16*'Catalogue'!$B$6*('Scenario inputs'!$U$16/'Scenario inputs'!$V$16/'Scenario inputs'!$W$16)+'Scenario inputs'!$S$16*'Catalogue'!$C$6+(1-'Scenario inputs'!$R$16-'Scenario inputs'!$S$16)*'Catalogue'!$D$6/'Scenario inputs'!$W$16)</x:f>
+        <x:v>20.833333333333336</x:v>
+      </x:c>
+      <x:c r="C16" s="130" t="n">
+        <x:f>B16*(1-'Scenario inputs'!$C$16)/(1+'Scenario inputs'!$B$16)</x:f>
+        <x:v>16.8732782369146</x:v>
+      </x:c>
+      <x:c r="D16" s="123" t="n">
+        <x:f>'Scenario inputs'!$R$16*('Scenario inputs'!$U$16/'Scenario inputs'!$V$16/'Scenario inputs'!$W$16)+'Scenario inputs'!$S$16+(1-'Scenario inputs'!$R$16-'Scenario inputs'!$S$16)/'Scenario inputs'!$W$16</x:f>
+        <x:v>0.08333333333333333</x:v>
+      </x:c>
+      <x:c r="E16" s="124" t="n">
+        <x:f>'Scenario inputs'!$Q$16*('Scenario inputs'!$R$16*'Catalogue'!$E$5*('Scenario inputs'!$U$16/'Scenario inputs'!$V$16/'Scenario inputs'!$W$16)+(1-'Scenario inputs'!$R$16)*'Catalogue'!$F$5)+(1-'Scenario inputs'!$Q$16)*('Scenario inputs'!$R$16*'Catalogue'!$E$6*('Scenario inputs'!$U$16/'Scenario inputs'!$V$16/'Scenario inputs'!$W$16)+(1-'Scenario inputs'!$R$16)*'Catalogue'!$F$6)</x:f>
+        <x:v>355</x:v>
+      </x:c>
+      <x:c r="F16" s="130" t="n">
+        <x:f>E16*'Scenario inputs'!$L$16*'Scenario inputs'!$M$16</x:f>
+        <x:v>3.5500000000000003</x:v>
+      </x:c>
+      <x:c r="G16" s="130" t="n">
+        <x:f>'Scenario inputs'!$Q$16*'Scenario inputs'!$N$16+(1-'Scenario inputs'!$Q$16)*'Scenario inputs'!$O$16</x:f>
+        <x:v>0.67</x:v>
+      </x:c>
+      <x:c r="H16" s="130" t="n">
+        <x:f>B16*('Scenario inputs'!$D$16+'Scenario inputs'!$E$16+'Scenario inputs'!$F$16+'Scenario inputs'!$X$16)</x:f>
+        <x:v>1.25</x:v>
+      </x:c>
+      <x:c r="I16" s="130" t="n">
+        <x:f>D16*('Scenario inputs'!$G$16+'Scenario inputs'!$Y$16*'Scenario inputs'!$Z$16)/'Scenario inputs'!$H$16</x:f>
+        <x:v>0.02235</x:v>
+      </x:c>
+      <x:c r="J16" s="130" t="n">
+        <x:f>B16*'Scenario inputs'!$I$16</x:f>
+        <x:v>0.10416666666666669</x:v>
+      </x:c>
+      <x:c r="K16" s="130" t="n">
+        <x:f>D16*'Scenario inputs'!$J$16*'Scenario inputs'!$K$16</x:f>
+        <x:v>0.0016666666666666666</x:v>
+      </x:c>
+      <x:c r="L16" s="131" t="n">
+        <x:f>SUM(F16:K16)</x:f>
+        <x:v>5.598183333333335</x:v>
+      </x:c>
+      <x:c r="M16" s="131" t="n">
+        <x:f>C16-L16</x:f>
+        <x:v>11.275094903581266</x:v>
+      </x:c>
+      <x:c r="N16" s="130" t="n">
+        <x:f>'Scenario inputs'!$P$16</x:f>
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="O16" s="124" t="n">
+        <x:f>IF(M16&lt;=0,"Not attainable",MAX(1,ROUNDUP(N16/M16,0)))</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="P16" s="124" t="n">
+        <x:f>IF(C16*(1-'Scenario inputs'!$T$16)-L16&lt;=0,"Not attainable",MAX(1,ROUNDUP(N16/(C16*(1-'Scenario inputs'!$T$16)-L16),0)))</x:f>
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="Q16" s="118" t="n">
+        <x:f>IF(C16=0,"Not defined",M16/C16)</x:f>
+        <x:v>0.668221951020408</x:v>
+      </x:c>
       <x:c r="R16" s="2"/>
       <x:c r="S16" s="2"/>
       <x:c r="T16" s="2"/>
@@ -15417,24 +15930,74 @@
       <x:c r="AJ16" s="2"/>
       <x:c r="AK16" s="2"/>
     </x:row>
-    <x:row r="17" ht="20" customHeight="1">
-      <x:c r="A17" s="2"/>
-      <x:c r="B17" s="2"/>
-      <x:c r="C17" s="2"/>
-      <x:c r="D17" s="2"/>
-      <x:c r="E17" s="2"/>
-      <x:c r="F17" s="2"/>
-      <x:c r="G17" s="2"/>
-      <x:c r="H17" s="2"/>
-      <x:c r="I17" s="2"/>
-      <x:c r="J17" s="2"/>
-      <x:c r="K17" s="2"/>
-      <x:c r="L17" s="2"/>
-      <x:c r="M17" s="2"/>
-      <x:c r="N17" s="2"/>
-      <x:c r="O17" s="2"/>
-      <x:c r="P17" s="2"/>
-      <x:c r="Q17" s="2"/>
+    <x:row r="17" ht="42" customHeight="1">
+      <x:c r="A17" s="30" t="str">
+        <x:v>Managed Payments Starter annual, full allowance</x:v>
+      </x:c>
+      <x:c r="B17" s="130" t="n">
+        <x:f>'Scenario inputs'!$Q$17*('Scenario inputs'!$R$17*'Catalogue'!$B$5*('Scenario inputs'!$U$17/'Scenario inputs'!$V$17/'Scenario inputs'!$W$17)+'Scenario inputs'!$S$17*'Catalogue'!$C$5+(1-'Scenario inputs'!$R$17-'Scenario inputs'!$S$17)*'Catalogue'!$D$5/'Scenario inputs'!$W$17)+(1-'Scenario inputs'!$Q$17)*('Scenario inputs'!$R$17*'Catalogue'!$B$6*('Scenario inputs'!$U$17/'Scenario inputs'!$V$17/'Scenario inputs'!$W$17)+'Scenario inputs'!$S$17*'Catalogue'!$C$6+(1-'Scenario inputs'!$R$17-'Scenario inputs'!$S$17)*'Catalogue'!$D$6/'Scenario inputs'!$W$17)</x:f>
+        <x:v>15.833333333333334</x:v>
+      </x:c>
+      <x:c r="C17" s="130" t="n">
+        <x:f>B17*(1-'Scenario inputs'!$C$17)/(1+'Scenario inputs'!$B$17)</x:f>
+        <x:v>12.823691460055098</x:v>
+      </x:c>
+      <x:c r="D17" s="123" t="n">
+        <x:f>'Scenario inputs'!$R$17*('Scenario inputs'!$U$17/'Scenario inputs'!$V$17/'Scenario inputs'!$W$17)+'Scenario inputs'!$S$17+(1-'Scenario inputs'!$R$17-'Scenario inputs'!$S$17)/'Scenario inputs'!$W$17</x:f>
+        <x:v>0.08333333333333333</x:v>
+      </x:c>
+      <x:c r="E17" s="124" t="n">
+        <x:f>'Scenario inputs'!$Q$17*('Scenario inputs'!$R$17*'Catalogue'!$E$5*('Scenario inputs'!$U$17/'Scenario inputs'!$V$17/'Scenario inputs'!$W$17)+(1-'Scenario inputs'!$R$17)*'Catalogue'!$F$5)+(1-'Scenario inputs'!$Q$17)*('Scenario inputs'!$R$17*'Catalogue'!$E$6*('Scenario inputs'!$U$17/'Scenario inputs'!$V$17/'Scenario inputs'!$W$17)+(1-'Scenario inputs'!$R$17)*'Catalogue'!$F$6)</x:f>
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="F17" s="130" t="n">
+        <x:f>E17*'Scenario inputs'!$L$17*'Scenario inputs'!$M$17</x:f>
+        <x:v>2.5</x:v>
+      </x:c>
+      <x:c r="G17" s="130" t="n">
+        <x:f>'Scenario inputs'!$Q$17*'Scenario inputs'!$N$17+(1-'Scenario inputs'!$Q$17)*'Scenario inputs'!$O$17</x:f>
+        <x:v>0.55</x:v>
+      </x:c>
+      <x:c r="H17" s="130" t="n">
+        <x:f>B17*('Scenario inputs'!$D$17+'Scenario inputs'!$E$17+'Scenario inputs'!$F$17+'Scenario inputs'!$X$17)</x:f>
+        <x:v>0.95</x:v>
+      </x:c>
+      <x:c r="I17" s="130" t="n">
+        <x:f>D17*('Scenario inputs'!$G$17+'Scenario inputs'!$Y$17*'Scenario inputs'!$Z$17)/'Scenario inputs'!$H$17</x:f>
+        <x:v>0.02235</x:v>
+      </x:c>
+      <x:c r="J17" s="130" t="n">
+        <x:f>B17*'Scenario inputs'!$I$17</x:f>
+        <x:v>0.07916666666666668</x:v>
+      </x:c>
+      <x:c r="K17" s="130" t="n">
+        <x:f>D17*'Scenario inputs'!$J$17*'Scenario inputs'!$K$17</x:f>
+        <x:v>0.0016666666666666666</x:v>
+      </x:c>
+      <x:c r="L17" s="131" t="n">
+        <x:f>SUM(F17:K17)</x:f>
+        <x:v>4.103183333333334</x:v>
+      </x:c>
+      <x:c r="M17" s="131" t="n">
+        <x:f>C17-L17</x:f>
+        <x:v>8.720508126721764</x:v>
+      </x:c>
+      <x:c r="N17" s="130" t="n">
+        <x:f>'Scenario inputs'!$P$17</x:f>
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="O17" s="124" t="n">
+        <x:f>IF(M17&lt;=0,"Not attainable",MAX(1,ROUNDUP(N17/M17,0)))</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="P17" s="124" t="n">
+        <x:f>IF(C17*(1-'Scenario inputs'!$T$17)-L17&lt;=0,"Not attainable",MAX(1,ROUNDUP(N17/(C17*(1-'Scenario inputs'!$T$17)-L17),0)))</x:f>
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="Q17" s="118" t="n">
+        <x:f>IF(C17=0,"Not defined",M17/C17)</x:f>
+        <x:v>0.6800310311493019</x:v>
+      </x:c>
       <x:c r="R17" s="2"/>
       <x:c r="S17" s="2"/>
       <x:c r="T17" s="2"/>

</xml_diff>